<commit_message>
Model1 dan 2 no result yet
</commit_message>
<xml_diff>
--- a/data/Laboratorium.xlsx
+++ b/data/Laboratorium.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Berkas UB\SKRIPSI\COATI\Coati_Optimization_University-Course-Schedulling\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A81ED4F-D89F-4D2F-BA48-CE70D821F6F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE4FD2F0-1F98-4A88-B8BE-C63FDAEBBDEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>G1.2</t>
   </si>
@@ -41,6 +41,15 @@
   </si>
   <si>
     <t>Kode Ruang</t>
+  </si>
+  <si>
+    <t>G1.7</t>
+  </si>
+  <si>
+    <t>G1.8</t>
+  </si>
+  <si>
+    <t>G1.9</t>
   </si>
 </sst>
 </file>
@@ -500,8 +509,12 @@
       <c r="X6" s="2"/>
     </row>
     <row r="7" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
+      <c r="A7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="2">
+        <v>1</v>
+      </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
@@ -526,8 +539,12 @@
       <c r="X7" s="2"/>
     </row>
     <row r="8" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
+      <c r="A8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="2">
+        <v>1</v>
+      </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
@@ -552,8 +569,12 @@
       <c r="X8" s="2"/>
     </row>
     <row r="9" spans="1:24" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
+      <c r="A9" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="2">
+        <v>1</v>
+      </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>

</xml_diff>